<commit_message>
Actualización automática: datos al 2026-06-14
</commit_message>
<xml_diff>
--- a/fondos-hencorp-rendimientos.xlsx
+++ b/fondos-hencorp-rendimientos.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-13)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AM4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AM5</f>
@@ -3158,7 +3158,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM2" t="n">
-        <v>233298679.38</v>
+        <v>233427759.85</v>
       </c>
     </row>
     <row r="3">
@@ -3264,7 +3264,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM3" t="n">
-        <v>683357555.03</v>
+        <v>683517826.35</v>
       </c>
     </row>
     <row r="4">
@@ -3497,7 +3497,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>233298679.38</v>
+        <v>233427759.85</v>
       </c>
     </row>
     <row r="12">
@@ -3516,7 +3516,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>683357555.03</v>
+        <v>683517826.35</v>
       </c>
     </row>
     <row r="13">
@@ -3886,7 +3886,7 @@
         <v>0.003951</v>
       </c>
       <c r="AM20" t="n">
-        <v>0.001484</v>
+        <v>0.00161</v>
       </c>
     </row>
     <row r="21">
@@ -3992,7 +3992,7 @@
         <v>-0.011932</v>
       </c>
       <c r="AM21" t="n">
-        <v>0.002813</v>
+        <v>0.003048</v>
       </c>
     </row>
     <row r="22">
@@ -4206,7 +4206,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-13) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-13)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14)</t>
         </is>
       </c>
     </row>
@@ -5580,7 +5580,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-13) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5757,6 +5757,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46186</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.17345303</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000125</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>233427759.85</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1043.95943762</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>683517826.35</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1217.11947157</v>
@@ -43862,7 +43880,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-13)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14)</t>
         </is>
       </c>
     </row>
@@ -44181,7 +44199,7 @@
         <v>1.17156713</v>
       </c>
       <c r="AM4" s="24" t="n">
-        <v>1.173306</v>
+        <v>1.17345303</v>
       </c>
     </row>
     <row r="5">
@@ -44292,7 +44310,7 @@
         <v>1040.78664211</v>
       </c>
       <c r="AM5" s="24" t="n">
-        <v>1043.71464992</v>
+        <v>1043.95943762</v>
       </c>
     </row>
     <row r="6">
@@ -44650,7 +44668,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-13)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14)</t>
         </is>
       </c>
     </row>
@@ -44969,7 +44987,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM4" s="25" t="n">
-        <v>233298679.38</v>
+        <v>233427759.85</v>
       </c>
     </row>
     <row r="5">
@@ -45080,7 +45098,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM5" s="25" t="n">
-        <v>683357555.03</v>
+        <v>683517826.35</v>
       </c>
     </row>
     <row r="6">
@@ -45410,7 +45428,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-06-14 (actualización 2026-06-13).</t>
+          <t>datos al 2026-06-14 (actualización 2026-06-14).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-06-15
</commit_message>
<xml_diff>
--- a/fondos-hencorp-rendimientos.xlsx
+++ b/fondos-hencorp-rendimientos.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-15)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AM4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AM5</f>
@@ -3158,7 +3158,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM2" t="n">
-        <v>233427759.85</v>
+        <v>233452068.94</v>
       </c>
     </row>
     <row r="3">
@@ -3264,7 +3264,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM3" t="n">
-        <v>683517826.35</v>
+        <v>683679976.38</v>
       </c>
     </row>
     <row r="4">
@@ -3497,7 +3497,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>233427759.85</v>
+        <v>233452068.94</v>
       </c>
     </row>
     <row r="12">
@@ -3516,7 +3516,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>683517826.35</v>
+        <v>683679976.38</v>
       </c>
     </row>
     <row r="13">
@@ -3886,7 +3886,7 @@
         <v>0.003951</v>
       </c>
       <c r="AM20" t="n">
-        <v>0.00161</v>
+        <v>0.001734</v>
       </c>
     </row>
     <row r="21">
@@ -3992,7 +3992,7 @@
         <v>-0.011932</v>
       </c>
       <c r="AM21" t="n">
-        <v>0.003048</v>
+        <v>0.003286</v>
       </c>
     </row>
     <row r="22">
@@ -4206,7 +4206,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-15) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-15)</t>
         </is>
       </c>
     </row>
@@ -5580,7 +5580,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-15) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5716,6 +5716,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46187</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.17359841</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000124</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>233452068.94</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1044.20709474</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000237</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>683679976.38</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1217.28420289</v>
@@ -43880,7 +43898,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-15)</t>
         </is>
       </c>
     </row>
@@ -44199,7 +44217,7 @@
         <v>1.17156713</v>
       </c>
       <c r="AM4" s="24" t="n">
-        <v>1.17345303</v>
+        <v>1.17359841</v>
       </c>
     </row>
     <row r="5">
@@ -44310,7 +44328,7 @@
         <v>1040.78664211</v>
       </c>
       <c r="AM5" s="24" t="n">
-        <v>1043.95943762</v>
+        <v>1044.20709474</v>
       </c>
     </row>
     <row r="6">
@@ -44668,7 +44686,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-14)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-14 (actualización 2026-06-15)</t>
         </is>
       </c>
     </row>
@@ -44987,7 +45005,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM4" s="25" t="n">
-        <v>233427759.85</v>
+        <v>233452068.94</v>
       </c>
     </row>
     <row r="5">
@@ -45098,7 +45116,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM5" s="25" t="n">
-        <v>683517826.35</v>
+        <v>683679976.38</v>
       </c>
     </row>
     <row r="6">
@@ -45428,7 +45446,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-06-14 (actualización 2026-06-14).</t>
+          <t>datos al 2026-06-14 (actualización 2026-06-15).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-06-18
</commit_message>
<xml_diff>
--- a/fondos-hencorp-rendimientos.xlsx
+++ b/fondos-hencorp-rendimientos.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-17)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-18)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AM4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AM5</f>
@@ -3158,7 +3158,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM2" t="n">
-        <v>230769696.12</v>
+        <v>230792730.94</v>
       </c>
     </row>
     <row r="3">
@@ -3264,7 +3264,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM3" t="n">
-        <v>679208026.05</v>
+        <v>679367942.36</v>
       </c>
     </row>
     <row r="4">
@@ -3497,7 +3497,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>230769696.12</v>
+        <v>230792730.94</v>
       </c>
     </row>
     <row r="12">
@@ -3516,7 +3516,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>679208026.05</v>
+        <v>679367942.36</v>
       </c>
     </row>
     <row r="13">
@@ -3886,7 +3886,7 @@
         <v>0.003951</v>
       </c>
       <c r="AM20" t="n">
-        <v>0.001982</v>
+        <v>0.002113</v>
       </c>
     </row>
     <row r="21">
@@ -3992,7 +3992,7 @@
         <v>-0.011932</v>
       </c>
       <c r="AM21" t="n">
-        <v>-0.003276</v>
+        <v>-0.003041</v>
       </c>
     </row>
     <row r="22">
@@ -4206,7 +4206,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-17) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-18) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-17)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-18)</t>
         </is>
       </c>
     </row>
@@ -5580,7 +5580,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-17) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-18) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5716,6 +5716,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46190</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.17404318</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>230792730.94</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1037.62118222</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>679367942.36</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1217.7783687</v>
@@ -44057,7 +44075,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-17)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-18)</t>
         </is>
       </c>
     </row>
@@ -44376,7 +44394,7 @@
         <v>1.17156713</v>
       </c>
       <c r="AM4" s="24" t="n">
-        <v>1.17388971</v>
+        <v>1.17404318</v>
       </c>
     </row>
     <row r="5">
@@ -44487,7 +44505,7 @@
         <v>1040.78664211</v>
       </c>
       <c r="AM5" s="24" t="n">
-        <v>1037.37693673</v>
+        <v>1037.62118222</v>
       </c>
     </row>
     <row r="6">
@@ -44845,7 +44863,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-17)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-17 (actualización 2026-06-18)</t>
         </is>
       </c>
     </row>
@@ -45164,7 +45182,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM4" s="25" t="n">
-        <v>230769696.12</v>
+        <v>230792730.94</v>
       </c>
     </row>
     <row r="5">
@@ -45275,7 +45293,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM5" s="25" t="n">
-        <v>679208026.05</v>
+        <v>679367942.36</v>
       </c>
     </row>
     <row r="6">
@@ -45605,7 +45623,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-06-17 (actualización 2026-06-17).</t>
+          <t>datos al 2026-06-17 (actualización 2026-06-18).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-06-21
</commit_message>
<xml_diff>
--- a/fondos-hencorp-rendimientos.xlsx
+++ b/fondos-hencorp-rendimientos.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-20)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AM4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AM5</f>
@@ -3158,7 +3158,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM2" t="n">
-        <v>225825185.81</v>
+        <v>225609882.21</v>
       </c>
     </row>
     <row r="3">
@@ -3264,7 +3264,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM3" t="n">
-        <v>679687878.15</v>
+        <v>679847855.39</v>
       </c>
     </row>
     <row r="4">
@@ -3497,7 +3497,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>225825185.81</v>
+        <v>225609882.21</v>
       </c>
     </row>
     <row r="12">
@@ -3516,7 +3516,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>679687878.15</v>
+        <v>679847855.39</v>
       </c>
     </row>
     <row r="13">
@@ -3886,7 +3886,7 @@
         <v>0.003951</v>
       </c>
       <c r="AM20" t="n">
-        <v>0.002373</v>
+        <v>0.002506</v>
       </c>
     </row>
     <row r="21">
@@ -3992,7 +3992,7 @@
         <v>-0.011932</v>
       </c>
       <c r="AM21" t="n">
-        <v>-0.002572</v>
+        <v>-0.002337</v>
       </c>
     </row>
     <row r="22">
@@ -4206,7 +4206,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-20) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-20)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21)</t>
         </is>
       </c>
     </row>
@@ -5580,7 +5580,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-20) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5757,6 +5757,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46193</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.17450272</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>225609882.21</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1038.3541693</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>679847855.39</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1218.27249207</v>
@@ -44275,7 +44293,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-20)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21)</t>
         </is>
       </c>
     </row>
@@ -44594,7 +44612,7 @@
         <v>1.17156713</v>
       </c>
       <c r="AM4" s="24" t="n">
-        <v>1.17434777</v>
+        <v>1.17450272</v>
       </c>
     </row>
     <row r="5">
@@ -44705,7 +44723,7 @@
         <v>1040.78664211</v>
       </c>
       <c r="AM5" s="24" t="n">
-        <v>1038.10983075</v>
+        <v>1038.3541693</v>
       </c>
     </row>
     <row r="6">
@@ -45063,7 +45081,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-20)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21)</t>
         </is>
       </c>
     </row>
@@ -45382,7 +45400,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM4" s="25" t="n">
-        <v>225825185.81</v>
+        <v>225609882.21</v>
       </c>
     </row>
     <row r="5">
@@ -45493,7 +45511,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM5" s="25" t="n">
-        <v>679687878.15</v>
+        <v>679847855.39</v>
       </c>
     </row>
     <row r="6">
@@ -45823,7 +45841,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-06-21 (actualización 2026-06-20).</t>
+          <t>datos al 2026-06-21 (actualización 2026-06-21).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-06-22
</commit_message>
<xml_diff>
--- a/fondos-hencorp-rendimientos.xlsx
+++ b/fondos-hencorp-rendimientos.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-22)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AM4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AM5</f>
@@ -3158,7 +3158,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM2" t="n">
-        <v>225609882.21</v>
+        <v>225660103.43</v>
       </c>
     </row>
     <row r="3">
@@ -3264,7 +3264,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM3" t="n">
-        <v>679847855.39</v>
+        <v>680007975.4299999</v>
       </c>
     </row>
     <row r="4">
@@ -3497,7 +3497,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>225609882.21</v>
+        <v>225660103.43</v>
       </c>
     </row>
     <row r="12">
@@ -3516,7 +3516,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>679847855.39</v>
+        <v>680007975.4299999</v>
       </c>
     </row>
     <row r="13">
@@ -3886,7 +3886,7 @@
         <v>0.003951</v>
       </c>
       <c r="AM20" t="n">
-        <v>0.002506</v>
+        <v>0.002638</v>
       </c>
     </row>
     <row r="21">
@@ -3992,7 +3992,7 @@
         <v>-0.011932</v>
       </c>
       <c r="AM21" t="n">
-        <v>-0.002337</v>
+        <v>-0.002102</v>
       </c>
     </row>
     <row r="22">
@@ -4206,7 +4206,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-22) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-22)</t>
         </is>
       </c>
     </row>
@@ -5580,7 +5580,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-22) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5716,6 +5716,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46194</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.17465766</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>225660103.43</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1038.59872595</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000236</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>680007975.4299999</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1218.43719033</v>
@@ -44293,7 +44311,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-22)</t>
         </is>
       </c>
     </row>
@@ -44612,7 +44630,7 @@
         <v>1.17156713</v>
       </c>
       <c r="AM4" s="24" t="n">
-        <v>1.17450272</v>
+        <v>1.17465766</v>
       </c>
     </row>
     <row r="5">
@@ -44723,7 +44741,7 @@
         <v>1040.78664211</v>
       </c>
       <c r="AM5" s="24" t="n">
-        <v>1038.3541693</v>
+        <v>1038.59872595</v>
       </c>
     </row>
     <row r="6">
@@ -45081,7 +45099,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-21)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Historico) | datos al 2026-06-21 (actualización 2026-06-22)</t>
         </is>
       </c>
     </row>
@@ -45400,7 +45418,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM4" s="25" t="n">
-        <v>225609882.21</v>
+        <v>225660103.43</v>
       </c>
     </row>
     <row r="5">
@@ -45511,7 +45529,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM5" s="25" t="n">
-        <v>679847855.39</v>
+        <v>680007975.4299999</v>
       </c>
     </row>
     <row r="6">
@@ -45841,7 +45859,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-06-21 (actualización 2026-06-21).</t>
+          <t>datos al 2026-06-21 (actualización 2026-06-22).</t>
         </is>
       </c>
     </row>

</xml_diff>